<commit_message>
Shipment 1 upload: keep both white jogger L SKUs home (170 units)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfDb7HTB9mKx6YmULmXMWR
</commit_message>
<xml_diff>
--- a/shipments/SFY_Shipment_1_Amazon_Upload.xlsx
+++ b/shipments/SFY_Shipment_1_Amazon_Upload.xlsx
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.97265625" defaultRowHeight="18"/>
   <cols>
     <col width="26.51171875" bestFit="1" customWidth="1" style="30" min="1" max="1"/>
@@ -2204,11 +2204,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KF-RYB4-6ZJD-FBA_L_Br</t>
+          <t>Jogger FW-FBA_S_Br</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>61034200</t>
+          <t>61046200</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -2230,11 +2230,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jogger FW-FBA_S_Br</t>
+          <t>Jogger FW-FBA_M_Br</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2256,11 +2256,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jogger FW-FBA_M_Br</t>
+          <t>Jogger F-FBA_S_Br</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -2282,11 +2282,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jogger FW-FBA_L_Br</t>
+          <t>Jogger F-FBA_M_Br</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -2308,11 +2308,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jogger F-FBA_S_Br</t>
+          <t>Jogger F-FBA_L_Br</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -2328,58 +2328,6 @@
         <v>5</v>
       </c>
       <c r="I31" t="n">
-        <v>1499</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Jogger F-FBA_M_Br</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>4</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>DEL4</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>61046200</t>
-        </is>
-      </c>
-      <c r="H32" t="n">
-        <v>5</v>
-      </c>
-      <c r="I32" t="n">
-        <v>1499</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Jogger F-FBA_L_Br</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>5</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>DEL4</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>61046200</t>
-        </is>
-      </c>
-      <c r="H33" t="n">
-        <v>5</v>
-      </c>
-      <c r="I33" t="n">
         <v>1499</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Shipment 1 upload: back to all 180 units (Seller labelling)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfDb7HTB9mKx6YmULmXMWR
</commit_message>
<xml_diff>
--- a/shipments/SFY_Shipment_1_Amazon_Upload.xlsx
+++ b/shipments/SFY_Shipment_1_Amazon_Upload.xlsx
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.97265625" defaultRowHeight="18"/>
   <cols>
     <col width="26.51171875" bestFit="1" customWidth="1" style="30" min="1" max="1"/>
@@ -2204,11 +2204,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Jogger FW-FBA_S_Br</t>
+          <t>KF-RYB4-6ZJD-FBA_L_Br</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>61046200</t>
+          <t>61034200</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -2230,11 +2230,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jogger FW-FBA_M_Br</t>
+          <t>Jogger FW-FBA_S_Br</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2256,11 +2256,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jogger F-FBA_S_Br</t>
+          <t>Jogger FW-FBA_M_Br</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -2282,11 +2282,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jogger F-FBA_M_Br</t>
+          <t>Jogger FW-FBA_L_Br</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -2308,11 +2308,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jogger F-FBA_L_Br</t>
+          <t>Jogger F-FBA_S_Br</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -2328,6 +2328,58 @@
         <v>5</v>
       </c>
       <c r="I31" t="n">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Jogger F-FBA_M_Br</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DEL4</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>61046200</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>5</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Jogger F-FBA_L_Br</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DEL4</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>61046200</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>5</v>
+      </c>
+      <c r="I33" t="n">
         <v>1499</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Shipment 1 upload: new white jogger L SKUs (_Br2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfDb7HTB9mKx6YmULmXMWR
</commit_message>
<xml_diff>
--- a/shipments/SFY_Shipment_1_Amazon_Upload.xlsx
+++ b/shipments/SFY_Shipment_1_Amazon_Upload.xlsx
@@ -2204,7 +2204,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KF-RYB4-6ZJD-FBA_L_Br</t>
+          <t>KF-RYB4-6ZJD-FBA_L_Br2</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2282,7 +2282,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jogger FW-FBA_L_Br</t>
+          <t>Jogger FW-FBA_L_Br2</t>
         </is>
       </c>
       <c r="B30" t="n">

</xml_diff>